<commit_message>
Arreglos formato y varios
</commit_message>
<xml_diff>
--- a/Copia Envases/ListaSalida.xlsx
+++ b/Copia Envases/ListaSalida.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$H$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,7 +490,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>190799</v>
+        <v>165639</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -525,19 +525,14 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>190810</v>
+        <v>165640</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>###</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>###</t>
+          <t>1670683 - 1670691</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -566,79 +561,117 @@
         <v>0</v>
       </c>
       <c r="B4" t="n">
-        <v>190810</v>
+        <v>218565</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1963101 - 1963102 - 1963104 - 1963107 - 1963108 - 1963109 - 1963110 - 1963111 - 1963112 - 1963113 - 1963114 - 1963115 - 1963116 - 1963117 - 1963118 - 1963119 - 1963120 - 1963121 - 1963122 - 1963123 - 1963125 - 1963127 - 1963129 - 1963130 - 1963131 - 1963132 - 1963133 - 1963135 - 1963138 - 1963139 - 1963140 - 1963141 - 1963142 - 1963143 - 1963144 - 1963145 - 1963146 - 1963147 - 1963150 - 1963152 - 1963153 - 1963155 - 1963156 - 1963159 - 1963161 - 1963162 - 1963165 - 1963166 - 1963170 - 1963171 - 1963172</t>
+          <t xml:space="preserve"> ![ 1744268 - 1823294 ]</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2222710 - 2222709 - 2222702 - 2222700 - 2222698 - 2222697 - 2222695 - 2222694 - 2222693 - 2222692 - 2222690 - 2222689 - 2222688 - 2222687 - 2222686 - 2222685 - 2222684 - 2222683 - 2222682 - 2222681 - 2222680 - 2222679 - 2222677 - 2222675 - 2222674 - 2222672 - 2222671 - 2222670 - 2222669 - 2222668 - 2222667 - 2222666 - 2222665 - 2222664 - 2222663 - 2222662 - 2222661 - 2222660 - 2222659 - 2222658 - 2222654 - 2222653 - 2222652 - 2222651 - 2222650 - 2222649 - 2222648 - 2222647 - 2222646 - 2222645 - 2222644 - 2222643 - 2222640 - 2222639 - 2222638 - 2222637 - 2222636 - 2222631 - 2222630 - 2222629 - 2222625 - 2222619 - 2222617 - 2222616 - 2222610 - 2222607 - 2222606 - 2222604 - 2222599 - 2222598 - 2222597 - 2222596 - 2222590 - 2222589 - 2222587 - 2222581 - 2222577 - 2222575 - 2222573 - 2222564 - 2222559 - 2222558 - 2222555 - 2222552 - 2222543 - 2222542 - 2222541 - 2222540 - 2222536 - 2222532 - 2222531 - 2222529 - 2222526 - 2222524 - 2222523 - 2222522 - 2222521 - 2222520 - 2222519 - 2222518</t>
+          <t>###</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>216319</t>
+          <t>###</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>PE21676/2025</t>
+          <t>###</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>PE - AGUAS PATAGONIA S.A - Coyhaique / Agua potable/bebida y Fuentes de captación</t>
+          <t>###</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>[M100C (57) (2222518)]</t>
+          <t>ERROR INICIO</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="n">
+        <v>220319</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ![ 2313194 - 2313195 ]</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>ERROR INICIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
         <v>0</v>
       </c>
-      <c r="B5" t="n">
-        <v>190810</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1963101 - 1963102 - 1963104 - 1963107 - 1963108 - 1963109 - 1963110 - 1963110 - 1963112 - 1963113 - 1963114 - 1963115 - 1963116 - 1963117 - 1963118 - 1963119 - 1963120 - 1963121 - 1963122 - 1963123 - 1963125 - 1963127 - 1963129 - 1963130 - 1963131 - 1963132 - 1963133 - 1963135 - 1963138 - 1963139 - 1963140 - 1963141 - 1963142 - 1963143 - 1963144 - 1963145 - 1963146 - 1963147 - 1963150 - 1963152 - 1963153 - 1963155 - 1963156 - 1963159 - 1963161 - 1963162 - 1963165 - 1963166 - 1963170 - 1963171 - 1963172</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2225070 - 2225069 - 2225068 - 2225064 - 2225063 - 2225062 - 2225058 - 2225057 - 2225056 - 2225052 - 2225044 - 2225043 - 2225042 - 2225041 - 2225040 - 2225039 - 2225038 - 2225033 - 2225032 - 2225031 - 2225030 - 2225029 - 2225028 - 2225027 - 2225026 - 2225024 - 2225022 - 2225021 - 2225020 - 2225019 - 2225017 - 2225016 - 2225014 - 2225013 - 2225012 - 2225011 - 2225010 - 2225007 - 2225006 - 2225005 - 2225004 - 2225003 - 2225002 - 2225001 - 2224998 - 2224997 - 2224996 - 2224995 - 2224991 - 2224990 - 2224989 - 2224988 - 2224986 - 2224984 - 2224982 - 2224981 - 2224980 - 2224979 - 2224978 - 2224977 - 2224976 - 2224974 - 2224973 - 2224972 - 2224971 - 2224970 - 2224969 - 2224967 - 2224963 - 2224961 - 2224959 - 2224957 - 2224947 - 2224946 - 2224945 - 2224944 - 2224942 - 2224941 - 2224940 - 2224938 - 2224936 - 2224935 - 2224934 - 2224933 - 2224932 - 2224931 - 2224929 - 2224928 - 2224927 - 2224924 - 2224920 - 2224919 - 2224917 - 2224912 - 2224907 - 2224905 - 2224902 - 2224892 - 2224889 - 2224888</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>216482</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PE21737/2025</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PE - AGUAS PATAGONIA S.A - Coyhaique / Agua potable/bebida y Fuentes de captación</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>[M100C (59) (2224888)]</t>
+      <c r="B6" t="n">
+        <v>218565</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>###</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>ERROR INICIO</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H5"/>
+  <autoFilter ref="A1:H6"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>